<commit_message>
docs(backend): 리포트 정정 — 이력 감지는 결정론적(recall 부족), chain_inclusion 재해석
진단 결과 반영:
- 이력 감지(history_mode)는 detect_history_intent 정규식으로만 결정되며(LLM은
  route만 담당) 결정론적이다. conflict 표현("바뀌었는가" 등)이 트리거에 안
  걸려 재현율 0% — "비결정적"이 아니라 감지 규칙의 recall 문제로 정정.
- chain_inclusion은 이력 라우팅 작동 지표가 아님을 명시: pair old/new 문구가
  검색 컨텍스트에 있는지만 검사하며 일반 하이브리드 검색으로도 통과한다
  (csbot B4: issue 행 "도입 여부" + decision 행 "정식 도입"). 따라서 audit
  미탐과 chain_inclusion=1.0은 모순이 아니라 서로 다른 것을 측정한 결과.
- 후속 태스크 재정의: TASK-008=이력 감지 개선(선행), TASK-009=supersede
  correctness(감지가 서야 유효).
- EVAL_REPORT.xlsx 한계·주석/컬럼설명 시트 동일 정정(export_report.py).
</commit_message>
<xml_diff>
--- a/docs/EVAL_REPORT.xlsx
+++ b/docs/EVAL_REPORT.xlsx
@@ -5624,10 +5624,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -5682,24 +5682,36 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>routing/chain</t>
+          <t>라우팅 감사</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>관측 지표(합격 조건 아님). 다수 문항 LLM 폴백이라 비결정 가능.</t>
+          <t>route(semantic/filter_lookup/overview)는 LLM 폴백이라 비결정 가능. 단 history_mode는 정규식이라 결정론적.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>chain_inclusion(modu E2-e2e)</t>
+          <t>이력 감지(history_mode)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.0 — 이력 체인 포함이 기대만큼 안 됨. TASK-007 범위 밖 후속 진단 대상.</t>
+          <t>정규식(detect_history_intent)으로만 켜짐(LLM은 route만). conflict 표현('바뀌었는가' 등)을 못 잡아 재현율 0% — 재현성 아닌 recall 문제. 개선=TASK-008(선행), supersede correctness=TASK-009.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>chain_inclusion</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>이력 라우팅 작동 지표가 아님 — pair old/new 문구가 검색 컨텍스트에 있는지만 검사(일반 검색으로도 통과, csbot 1.0이 그 경우).</t>
         </is>
       </c>
     </row>
@@ -5825,7 +5837,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>이력 체인 포함률(E2, 기대 pair 문구 포함) — 높을수록 좋음</t>
+          <t>pair old/new 문구가 검색 컨텍스트에 포함됐는지 검사(E2) — 이력 라우팅 작동 여부가 아님(일반 검색으로도 통과)</t>
         </is>
       </c>
     </row>

</xml_diff>